<commit_message>
Remove audit extraction script and output files: clean up comprehensive answer extraction validation analysis including Python audit script, 71,049-record item-level CSV, model summary statistics, log accuracy verification, and GPT empty response documentation
</commit_message>
<xml_diff>
--- a/Candidate_analysis/outputs/mann_whitney_LLM_vs_candidates.xlsx
+++ b/Candidate_analysis/outputs/mann_whitney_LLM_vs_candidates.xlsx
@@ -1664,7 +1664,7 @@
         <v>0.0000000000000204976410463988</v>
       </c>
       <c r="J32" t="n">
-        <v>0.000000000000143483487324792</v>
+        <v>0.000000000000122985846278393</v>
       </c>
       <c r="K32" t="s">
         <v>14</v>
@@ -1702,7 +1702,7 @@
         <v>0.00000000000000598703003526595</v>
       </c>
       <c r="J33" t="n">
-        <v>0.0000000000000478962402821276</v>
+        <v>0.0000000000000419092102468616</v>
       </c>
       <c r="K33" t="s">
         <v>14</v>
@@ -1734,13 +1734,13 @@
         <v>78.5</v>
       </c>
       <c r="H34" t="n">
-        <v>788955.5</v>
+        <v>799043</v>
       </c>
       <c r="I34" t="n">
-        <v>0.0000000000000248535713217188</v>
+        <v>0.00000000000000336692302229569</v>
       </c>
       <c r="J34" t="n">
-        <v>0.000000000000149121427930313</v>
+        <v>0.0000000000000269353841783655</v>
       </c>
       <c r="K34" t="s">
         <v>14</v>
@@ -2418,13 +2418,13 @@
         <v>80.5</v>
       </c>
       <c r="H52" t="n">
-        <v>680640</v>
+        <v>682112</v>
       </c>
       <c r="I52" t="n">
-        <v>0.000000000000000000646144723735494</v>
+        <v>0.000000000000000000428103610965252</v>
       </c>
       <c r="J52" t="n">
-        <v>0.00000000000000000581530251361945</v>
+        <v>0.00000000000000000385293249868727</v>
       </c>
       <c r="K52" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
Update item-level accuracy data for MedGemma 1.5-4B-Q8_0 question 116 (2021): correct response rate increases from 0.16 to 0.18, propagating minor numerical changes through statistical outputs including Kruskal-Wallis effect sizes, pairwise comparisons, Mann-Whitney effect sizes, quantization comparisons, and group-level accuracy summaries
</commit_message>
<xml_diff>
--- a/Candidate_analysis/outputs/mann_whitney_LLM_vs_candidates.xlsx
+++ b/Candidate_analysis/outputs/mann_whitney_LLM_vs_candidates.xlsx
@@ -1734,13 +1734,13 @@
         <v>78.5</v>
       </c>
       <c r="H34" t="n">
-        <v>799043</v>
+        <v>799328.5</v>
       </c>
       <c r="I34" t="n">
-        <v>0.00000000000000336692302229569</v>
+        <v>0.00000000000000317878520073589</v>
       </c>
       <c r="J34" t="n">
-        <v>0.0000000000000269353841783655</v>
+        <v>0.0000000000000254302816058871</v>
       </c>
       <c r="K34" t="s">
         <v>14</v>

</xml_diff>